<commit_message>
Temporarily remove time adjusted capacity factor multiplier
</commit_message>
<xml_diff>
--- a/InputData/elec/TACFMfPBTY/Time Adjusted Capacity Factor Multiplier for Plants Built This Year.xlsx
+++ b/InputData/elec/TACFMfPBTY/Time Adjusted Capacity Factor Multiplier for Plants Built This Year.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\TACFMfPBTY\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C6D6DBE-C177-4B4E-AB68-7539FB6A2B52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23C9B1BD-DF80-4C34-B336-D9182DEC238D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24120" yWindow="6690" windowWidth="24240" windowHeight="13020" xr2:uid="{EBD0EF52-E4BC-4E99-950E-1B8A93112F65}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{EBD0EF52-E4BC-4E99-950E-1B8A93112F65}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="2" r:id="rId1"/>
@@ -253,7 +253,7 @@
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -272,7 +272,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -640,17 +639,17 @@
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A10" s="10" t="s">
+      <c r="A10" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A11" s="10" t="s">
+      <c r="A11" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A12" s="10" t="s">
+      <c r="A12" t="s">
         <v>9</v>
       </c>
     </row>
@@ -746,7 +745,7 @@
         <v>17</v>
       </c>
       <c r="B2">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="C2" s="7"/>
       <c r="D2" s="7"/>
@@ -777,7 +776,7 @@
         <v>18</v>
       </c>
       <c r="B3">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
@@ -808,7 +807,7 @@
         <v>19</v>
       </c>
       <c r="B4">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
@@ -839,7 +838,7 @@
         <v>20</v>
       </c>
       <c r="B5">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="C5" s="7"/>
       <c r="D5" s="7"/>
@@ -870,7 +869,7 @@
         <v>21</v>
       </c>
       <c r="B6">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
@@ -901,7 +900,7 @@
         <v>22</v>
       </c>
       <c r="B7">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -932,7 +931,7 @@
         <v>23</v>
       </c>
       <c r="B8">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
@@ -963,7 +962,7 @@
         <v>24</v>
       </c>
       <c r="B9">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
@@ -994,7 +993,7 @@
         <v>25</v>
       </c>
       <c r="B10">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="7"/>
@@ -1025,7 +1024,7 @@
         <v>26</v>
       </c>
       <c r="B11">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="7"/>
@@ -1056,7 +1055,7 @@
         <v>27</v>
       </c>
       <c r="B12">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="C12" s="7"/>
       <c r="D12" s="7"/>
@@ -1087,7 +1086,7 @@
         <v>28</v>
       </c>
       <c r="B13">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="7"/>
@@ -1118,7 +1117,7 @@
         <v>29</v>
       </c>
       <c r="B14">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="C14" s="7"/>
       <c r="D14" s="7"/>
@@ -1149,7 +1148,7 @@
         <v>30</v>
       </c>
       <c r="B15">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="C15" s="7"/>
       <c r="D15" s="7"/>
@@ -1180,7 +1179,7 @@
         <v>31</v>
       </c>
       <c r="B16">
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
@@ -1188,7 +1187,7 @@
         <v>32</v>
       </c>
       <c r="B17">
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
@@ -1196,7 +1195,7 @@
         <v>33</v>
       </c>
       <c r="B18">
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
@@ -1204,7 +1203,7 @@
         <v>34</v>
       </c>
       <c r="B19">
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
@@ -1212,7 +1211,7 @@
         <v>35</v>
       </c>
       <c r="B20">
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
@@ -1220,7 +1219,7 @@
         <v>36</v>
       </c>
       <c r="B21">
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
@@ -1228,7 +1227,7 @@
         <v>37</v>
       </c>
       <c r="B22">
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.35">
@@ -1236,23 +1235,23 @@
         <v>38</v>
       </c>
       <c r="B23">
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A24" s="11" t="s">
+      <c r="A24" s="10" t="s">
         <v>39</v>
       </c>
       <c r="B24">
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A25" s="11" t="s">
+      <c r="A25" s="10" t="s">
         <v>40</v>
       </c>
       <c r="B25">
-        <v>0.5</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add time adjustment multipliers into SYSHECF and reset TACFMfPBTY to 0.5
</commit_message>
<xml_diff>
--- a/InputData/elec/TACFMfPBTY/Time Adjusted Capacity Factor Multiplier for Plants Built This Year.xlsx
+++ b/InputData/elec/TACFMfPBTY/Time Adjusted Capacity Factor Multiplier for Plants Built This Year.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\TACFMfPBTY\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23C9B1BD-DF80-4C34-B336-D9182DEC238D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2F4036F-DB6E-4E4C-B822-CCA3A720CD85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{EBD0EF52-E4BC-4E99-950E-1B8A93112F65}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{EBD0EF52-E4BC-4E99-950E-1B8A93112F65}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="2" r:id="rId1"/>
@@ -745,7 +745,7 @@
         <v>17</v>
       </c>
       <c r="B2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="C2" s="7"/>
       <c r="D2" s="7"/>
@@ -776,7 +776,7 @@
         <v>18</v>
       </c>
       <c r="B3">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
@@ -807,7 +807,7 @@
         <v>19</v>
       </c>
       <c r="B4">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
@@ -838,7 +838,7 @@
         <v>20</v>
       </c>
       <c r="B5">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="C5" s="7"/>
       <c r="D5" s="7"/>
@@ -869,7 +869,7 @@
         <v>21</v>
       </c>
       <c r="B6">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
@@ -900,7 +900,7 @@
         <v>22</v>
       </c>
       <c r="B7">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -931,7 +931,7 @@
         <v>23</v>
       </c>
       <c r="B8">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
@@ -962,7 +962,7 @@
         <v>24</v>
       </c>
       <c r="B9">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
@@ -993,7 +993,7 @@
         <v>25</v>
       </c>
       <c r="B10">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="7"/>
@@ -1024,7 +1024,7 @@
         <v>26</v>
       </c>
       <c r="B11">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="7"/>
@@ -1055,7 +1055,7 @@
         <v>27</v>
       </c>
       <c r="B12">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="C12" s="7"/>
       <c r="D12" s="7"/>
@@ -1086,7 +1086,7 @@
         <v>28</v>
       </c>
       <c r="B13">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="7"/>
@@ -1117,7 +1117,7 @@
         <v>29</v>
       </c>
       <c r="B14">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="C14" s="7"/>
       <c r="D14" s="7"/>
@@ -1148,7 +1148,7 @@
         <v>30</v>
       </c>
       <c r="B15">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="C15" s="7"/>
       <c r="D15" s="7"/>
@@ -1179,7 +1179,7 @@
         <v>31</v>
       </c>
       <c r="B16">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
@@ -1187,7 +1187,7 @@
         <v>32</v>
       </c>
       <c r="B17">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
@@ -1195,7 +1195,7 @@
         <v>33</v>
       </c>
       <c r="B18">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
@@ -1203,7 +1203,7 @@
         <v>34</v>
       </c>
       <c r="B19">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
@@ -1211,7 +1211,7 @@
         <v>35</v>
       </c>
       <c r="B20">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
@@ -1219,7 +1219,7 @@
         <v>36</v>
       </c>
       <c r="B21">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
@@ -1227,7 +1227,7 @@
         <v>37</v>
       </c>
       <c r="B22">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.35">
@@ -1235,7 +1235,7 @@
         <v>38</v>
       </c>
       <c r="B23">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.35">
@@ -1243,7 +1243,7 @@
         <v>39</v>
       </c>
       <c r="B24">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.35">
@@ -1251,7 +1251,7 @@
         <v>40</v>
       </c>
       <c r="B25">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Turns TACFMfPBTY back on (for calibration; was originally turned off due to y/o/y build oscillations)
</commit_message>
<xml_diff>
--- a/InputData/elec/TACFMfPBTY/Time Adjusted Capacity Factor Multiplier for Plants Built This Year.xlsx
+++ b/InputData/elec/TACFMfPBTY/Time Adjusted Capacity Factor Multiplier for Plants Built This Year.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\elec\TACFMfPBTY\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{040D0086-ECBF-44EA-908E-719592D378A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C20CE74-59A4-4704-959B-BD89C6DD7FCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2660" yWindow="2660" windowWidth="14400" windowHeight="8170" activeTab="1" xr2:uid="{EBD0EF52-E4BC-4E99-950E-1B8A93112F65}"/>
+    <workbookView xWindow="20" yWindow="740" windowWidth="19180" windowHeight="11260" activeTab="1" xr2:uid="{EBD0EF52-E4BC-4E99-950E-1B8A93112F65}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="2" r:id="rId1"/>
@@ -593,17 +593,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3FA4BC6-E9B6-4A5C-B81E-1C82F1EFD636}">
   <dimension ref="A1:C33"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="15.81640625" customWidth="1"/>
+    <col min="2" max="2" width="15.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -611,82 +611,82 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>2</v>
       </c>
       <c r="B5" s="3"/>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>4</v>
       </c>
       <c r="B7" s="4"/>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B31" s="9"/>
       <c r="C31" s="9"/>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B32" s="8"/>
       <c r="C32" s="8"/>
     </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B33" s="8"/>
       <c r="C33" s="8"/>
     </row>
@@ -702,14 +702,14 @@
     <tabColor rgb="FF002060"/>
   </sheetPr>
   <dimension ref="A1:Y25"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.54296875" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" customWidth="1"/>
     <col min="2" max="2" width="12" bestFit="1" customWidth="1"/>
-    <col min="3" max="25" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="25" width="10.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>16</v>
       </c>
@@ -740,7 +740,7 @@
       <c r="X1" s="6"/>
       <c r="Y1" s="6"/>
     </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>17</v>
       </c>
@@ -771,7 +771,7 @@
       <c r="X2" s="7"/>
       <c r="Y2" s="7"/>
     </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -802,7 +802,7 @@
       <c r="X3" s="7"/>
       <c r="Y3" s="7"/>
     </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>19</v>
       </c>
@@ -833,7 +833,7 @@
       <c r="X4" s="7"/>
       <c r="Y4" s="7"/>
     </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>20</v>
       </c>
@@ -864,7 +864,7 @@
       <c r="X5" s="7"/>
       <c r="Y5" s="7"/>
     </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -895,12 +895,12 @@
       <c r="X6" s="7"/>
       <c r="Y6" s="7"/>
     </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>22</v>
       </c>
       <c r="B7">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -926,12 +926,12 @@
       <c r="X7" s="7"/>
       <c r="Y7" s="7"/>
     </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>23</v>
       </c>
       <c r="B8">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
@@ -957,7 +957,7 @@
       <c r="X8" s="7"/>
       <c r="Y8" s="7"/>
     </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>24</v>
       </c>
@@ -988,7 +988,7 @@
       <c r="X9" s="7"/>
       <c r="Y9" s="7"/>
     </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>25</v>
       </c>
@@ -1019,7 +1019,7 @@
       <c r="X10" s="7"/>
       <c r="Y10" s="7"/>
     </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>26</v>
       </c>
@@ -1050,7 +1050,7 @@
       <c r="X11" s="7"/>
       <c r="Y11" s="7"/>
     </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>27</v>
       </c>
@@ -1081,7 +1081,7 @@
       <c r="X12" s="7"/>
       <c r="Y12" s="7"/>
     </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>28</v>
       </c>
@@ -1112,7 +1112,7 @@
       <c r="X13" s="7"/>
       <c r="Y13" s="7"/>
     </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>29</v>
       </c>
@@ -1143,7 +1143,7 @@
       <c r="X14" s="7"/>
       <c r="Y14" s="7"/>
     </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>30</v>
       </c>
@@ -1174,7 +1174,7 @@
       <c r="X15" s="7"/>
       <c r="Y15" s="7"/>
     </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>31</v>
       </c>
@@ -1182,7 +1182,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>32</v>
       </c>
@@ -1190,7 +1190,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>33</v>
       </c>
@@ -1198,7 +1198,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>34</v>
       </c>
@@ -1206,7 +1206,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>35</v>
       </c>
@@ -1214,7 +1214,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>36</v>
       </c>
@@ -1222,7 +1222,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>37</v>
       </c>
@@ -1230,7 +1230,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>38</v>
       </c>
@@ -1238,7 +1238,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="10" t="s">
         <v>39</v>
       </c>
@@ -1246,7 +1246,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="10" t="s">
         <v>40</v>
       </c>

</xml_diff>

<commit_message>
Reset TACFMfPBTY to 0.5
</commit_message>
<xml_diff>
--- a/InputData/elec/TACFMfPBTY/Time Adjusted Capacity Factor Multiplier for Plants Built This Year.xlsx
+++ b/InputData/elec/TACFMfPBTY/Time Adjusted Capacity Factor Multiplier for Plants Built This Year.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\elec\TACFMfPBTY\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\TACFMfPBTY\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C20CE74-59A4-4704-959B-BD89C6DD7FCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F04370D5-5FEC-40DB-8F4A-F2658DBC862A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="740" windowWidth="19180" windowHeight="11260" activeTab="1" xr2:uid="{EBD0EF52-E4BC-4E99-950E-1B8A93112F65}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{EBD0EF52-E4BC-4E99-950E-1B8A93112F65}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="2" r:id="rId1"/>
@@ -745,7 +745,7 @@
         <v>17</v>
       </c>
       <c r="B2">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="C2" s="7"/>
       <c r="D2" s="7"/>
@@ -776,7 +776,7 @@
         <v>18</v>
       </c>
       <c r="B3">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
@@ -807,7 +807,7 @@
         <v>19</v>
       </c>
       <c r="B4">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
@@ -838,7 +838,7 @@
         <v>20</v>
       </c>
       <c r="B5">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="C5" s="7"/>
       <c r="D5" s="7"/>
@@ -869,7 +869,7 @@
         <v>21</v>
       </c>
       <c r="B6">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
@@ -900,7 +900,7 @@
         <v>22</v>
       </c>
       <c r="B7">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -931,7 +931,7 @@
         <v>23</v>
       </c>
       <c r="B8">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
@@ -962,7 +962,7 @@
         <v>24</v>
       </c>
       <c r="B9">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
@@ -993,7 +993,7 @@
         <v>25</v>
       </c>
       <c r="B10">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="7"/>
@@ -1024,7 +1024,7 @@
         <v>26</v>
       </c>
       <c r="B11">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="7"/>
@@ -1055,7 +1055,7 @@
         <v>27</v>
       </c>
       <c r="B12">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="C12" s="7"/>
       <c r="D12" s="7"/>
@@ -1086,7 +1086,7 @@
         <v>28</v>
       </c>
       <c r="B13">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="7"/>
@@ -1117,7 +1117,7 @@
         <v>29</v>
       </c>
       <c r="B14">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="C14" s="7"/>
       <c r="D14" s="7"/>
@@ -1148,7 +1148,7 @@
         <v>30</v>
       </c>
       <c r="B15">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="C15" s="7"/>
       <c r="D15" s="7"/>
@@ -1179,7 +1179,7 @@
         <v>31</v>
       </c>
       <c r="B16">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -1187,7 +1187,7 @@
         <v>32</v>
       </c>
       <c r="B17">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -1195,7 +1195,7 @@
         <v>33</v>
       </c>
       <c r="B18">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -1203,7 +1203,7 @@
         <v>34</v>
       </c>
       <c r="B19">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -1211,7 +1211,7 @@
         <v>35</v>
       </c>
       <c r="B20">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -1219,7 +1219,7 @@
         <v>36</v>
       </c>
       <c r="B21">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -1227,7 +1227,7 @@
         <v>37</v>
       </c>
       <c r="B22">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -1235,7 +1235,7 @@
         <v>38</v>
       </c>
       <c r="B23">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -1243,7 +1243,7 @@
         <v>39</v>
       </c>
       <c r="B24">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -1251,7 +1251,7 @@
         <v>40</v>
       </c>
       <c r="B25">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>